<commit_message>
Voy a agregar nuevas metas dic Prueba
</commit_message>
<xml_diff>
--- a/data/metas/Metas nov.xlsx
+++ b/data/metas/Metas nov.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vladimir\Documents\Reportes\track\TRACK BI\data\metas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4304BF88-FCE7-4974-818B-CE1B35B1A252}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B93E017C-8C2B-4309-BA96-CBC2BB349397}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{25CE6252-27A9-4B41-ABF1-E4554C54E68E}"/>
+    <workbookView xWindow="-28908" yWindow="-108" windowWidth="29016" windowHeight="15696" xr2:uid="{25CE6252-27A9-4B41-ABF1-E4554C54E68E}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="35">
   <si>
     <t>VILLAS DEL REY</t>
   </si>
@@ -149,7 +149,7 @@
     <numFmt numFmtId="164" formatCode="_-[$$-80A]* #,##0_-;\-[$$-80A]* #,##0_-;_-[$$-80A]* &quot;-&quot;??_-;_-@"/>
     <numFmt numFmtId="165" formatCode="_-&quot;$&quot;* #,##0_-;\-&quot;$&quot;* #,##0_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -184,6 +184,18 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -193,7 +205,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -236,11 +248,40 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFECECEC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -262,48 +303,46 @@
     <xf numFmtId="1" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="13">
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FF000000"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF000000"/>
-        </right>
-        <top/>
-        <bottom style="thin">
-          <color rgb="FF000000"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -395,6 +434,40 @@
         <scheme val="none"/>
       </font>
       <numFmt numFmtId="164" formatCode="_-[$$-80A]* #,##0_-;\-[$$-80A]* #,##0_-;_-[$$-80A]* &quot;-&quot;??_-;_-@"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top/>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color rgb="FF000000"/>
@@ -659,8 +732,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{270C0CE8-2C9D-4E45-89F3-304CDC43FD91}" name="Tabla1" displayName="Tabla1" ref="A2:M24" totalsRowShown="0" tableBorderDxfId="12">
-  <autoFilter ref="A2:M24" xr:uid="{270C0CE8-2C9D-4E45-89F3-304CDC43FD91}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{270C0CE8-2C9D-4E45-89F3-304CDC43FD91}" name="Tabla1" displayName="Tabla1" ref="A2:M46" totalsRowShown="0" tableBorderDxfId="12">
+  <autoFilter ref="A2:M46" xr:uid="{270C0CE8-2C9D-4E45-89F3-304CDC43FD91}"/>
   <tableColumns count="13">
     <tableColumn id="1" xr3:uid="{77AEC5E1-75A8-4D26-B7C6-FEB178F6E1C1}" name="Sucursales" dataDxfId="11"/>
     <tableColumn id="2" xr3:uid="{7462DAAF-6DB4-4405-8508-73A33ADDFB4F}" name="Meta FAYCGO " dataDxfId="10"/>
@@ -669,14 +742,14 @@
     <tableColumn id="5" xr3:uid="{66334719-0049-403A-B612-EEE7CDCFD91E}" name="Meta de clientes nuevos" dataDxfId="7"/>
     <tableColumn id="11" xr3:uid="{3747F394-BC92-4DF9-82AB-77A6FF06F22A}" name="Meta reactivaciones" dataDxfId="6"/>
     <tableColumn id="12" xr3:uid="{C523342F-9057-4D3B-8835-7F6D9A6E1EFD}" name="ARPU" dataDxfId="5"/>
-    <tableColumn id="13" xr3:uid="{A191A5EF-FD11-4DA3-ABF9-6BFF96600642}" name="Meta bajas" dataDxfId="0"/>
-    <tableColumn id="6" xr3:uid="{E4A3EC2D-E11C-4CA1-BFB3-B808B639E6CC}" name="Bebidas" dataDxfId="4">
+    <tableColumn id="13" xr3:uid="{A191A5EF-FD11-4DA3-ABF9-6BFF96600642}" name="Meta bajas" dataDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{E4A3EC2D-E11C-4CA1-BFB3-B808B639E6CC}" name="Bebidas" dataDxfId="3">
       <calculatedColumnFormula>B3*0.07</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{019A4BB1-5D06-464D-AA21-8078EFD6DBF4}" name="Artículos" dataDxfId="3">
+    <tableColumn id="7" xr3:uid="{019A4BB1-5D06-464D-AA21-8078EFD6DBF4}" name="Artículos" dataDxfId="2">
       <calculatedColumnFormula>(B3*0.013)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{70BCCEC0-77FB-4C5B-A333-BAA74285D0C7}" name="Tienda" dataDxfId="2">
+    <tableColumn id="8" xr3:uid="{70BCCEC0-77FB-4C5B-A333-BAA74285D0C7}" name="Tienda" dataDxfId="1">
       <calculatedColumnFormula>I3+J3</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="9" xr3:uid="{5072CA0F-EA14-4D3C-A062-1A5ABD714150}" name="Año"/>
@@ -983,7 +1056,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{404D95DA-BDF5-4CE9-B38E-D0639C2B77E5}">
-  <dimension ref="A2:M24"/>
+  <dimension ref="A2:M46"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21.109375" bestFit="1" customWidth="1"/>
@@ -1065,11 +1138,11 @@
         <v>287</v>
       </c>
       <c r="I3" s="4">
-        <f>B3*0.07</f>
+        <f t="shared" ref="I3:I24" si="0">B3*0.07</f>
         <v>54881.890000000007</v>
       </c>
       <c r="J3" s="5">
-        <f>(B3*0.013)</f>
+        <f t="shared" ref="J3:J24" si="1">(B3*0.013)</f>
         <v>10192.350999999999</v>
       </c>
       <c r="K3" s="6">
@@ -1109,15 +1182,15 @@
         <v>198</v>
       </c>
       <c r="I4" s="4">
-        <f>B4*0.07</f>
+        <f t="shared" si="0"/>
         <v>47539.100000000006</v>
       </c>
       <c r="J4" s="5">
-        <f>(B4*0.013)</f>
+        <f t="shared" si="1"/>
         <v>8828.6899999999987</v>
       </c>
       <c r="K4" s="6">
-        <f t="shared" ref="K4:K24" si="0">I4+J4</f>
+        <f t="shared" ref="K4:K24" si="2">I4+J4</f>
         <v>56367.790000000008</v>
       </c>
       <c r="L4">
@@ -1153,15 +1226,15 @@
         <v>226</v>
       </c>
       <c r="I5" s="4">
-        <f>B5*0.07</f>
+        <f t="shared" si="0"/>
         <v>58825.200000000004</v>
       </c>
       <c r="J5" s="5">
-        <f>(B5*0.013)</f>
+        <f t="shared" si="1"/>
         <v>10924.68</v>
       </c>
       <c r="K5" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>69749.88</v>
       </c>
       <c r="L5">
@@ -1197,15 +1270,15 @@
         <v>225</v>
       </c>
       <c r="I6" s="4">
-        <f>B6*0.07</f>
+        <f t="shared" si="0"/>
         <v>55701.73</v>
       </c>
       <c r="J6" s="5">
-        <f>(B6*0.013)</f>
+        <f t="shared" si="1"/>
         <v>10344.607</v>
       </c>
       <c r="K6" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>66046.337</v>
       </c>
       <c r="L6">
@@ -1241,15 +1314,15 @@
         <v>403</v>
       </c>
       <c r="I7" s="4">
-        <f>B7*0.07</f>
+        <f t="shared" si="0"/>
         <v>78682.8</v>
       </c>
       <c r="J7" s="5">
-        <f>(B7*0.013)</f>
+        <f t="shared" si="1"/>
         <v>14612.519999999999</v>
       </c>
       <c r="K7" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>93295.32</v>
       </c>
       <c r="L7">
@@ -1285,15 +1358,15 @@
         <v>221</v>
       </c>
       <c r="I8" s="4">
-        <f>B8*0.07</f>
+        <f t="shared" si="0"/>
         <v>52070.340000000004</v>
       </c>
       <c r="J8" s="5">
-        <f>(B8*0.013)</f>
+        <f t="shared" si="1"/>
         <v>9670.2060000000001</v>
       </c>
       <c r="K8" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>61740.546000000002</v>
       </c>
       <c r="L8">
@@ -1329,15 +1402,15 @@
         <v>236</v>
       </c>
       <c r="I9" s="4">
-        <f>B9*0.07</f>
+        <f t="shared" si="0"/>
         <v>46803.890000000007</v>
       </c>
       <c r="J9" s="5">
-        <f>(B9*0.013)</f>
+        <f t="shared" si="1"/>
         <v>8692.1509999999998</v>
       </c>
       <c r="K9" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>55496.041000000005</v>
       </c>
       <c r="L9">
@@ -1373,15 +1446,15 @@
         <v>419</v>
       </c>
       <c r="I10" s="4">
-        <f>B10*0.07</f>
+        <f t="shared" si="0"/>
         <v>65562</v>
       </c>
       <c r="J10" s="5">
-        <f>(B10*0.013)</f>
+        <f t="shared" si="1"/>
         <v>12175.8</v>
       </c>
       <c r="K10" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>77737.8</v>
       </c>
       <c r="L10">
@@ -1417,15 +1490,15 @@
         <v>526</v>
       </c>
       <c r="I11" s="4">
-        <f>B11*0.07</f>
+        <f t="shared" si="0"/>
         <v>111677.44000000002</v>
       </c>
       <c r="J11" s="5">
-        <f>(B11*0.013)</f>
+        <f t="shared" si="1"/>
         <v>20740.095999999998</v>
       </c>
       <c r="K11" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>132417.53600000002</v>
       </c>
       <c r="L11">
@@ -1461,15 +1534,15 @@
         <v>154</v>
       </c>
       <c r="I12" s="4">
-        <f>B12*0.07</f>
+        <f t="shared" si="0"/>
         <v>28170.870000000003</v>
       </c>
       <c r="J12" s="5">
-        <f>(B12*0.013)</f>
+        <f t="shared" si="1"/>
         <v>5231.7330000000002</v>
       </c>
       <c r="K12" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>33402.603000000003</v>
       </c>
       <c r="L12">
@@ -1505,15 +1578,15 @@
         <v>391</v>
       </c>
       <c r="I13" s="4">
-        <f>B13*0.07</f>
+        <f t="shared" si="0"/>
         <v>79259.950000000012</v>
       </c>
       <c r="J13" s="5">
-        <f>(B13*0.013)</f>
+        <f t="shared" si="1"/>
         <v>14719.705</v>
       </c>
       <c r="K13" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>93979.655000000013</v>
       </c>
       <c r="L13">
@@ -1549,15 +1622,15 @@
         <v>377</v>
       </c>
       <c r="I14" s="4">
-        <f>B14*0.07</f>
+        <f t="shared" si="0"/>
         <v>76499.780000000013</v>
       </c>
       <c r="J14" s="5">
-        <f>(B14*0.013)</f>
+        <f t="shared" si="1"/>
         <v>14207.101999999999</v>
       </c>
       <c r="K14" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>90706.882000000012</v>
       </c>
       <c r="L14">
@@ -1593,15 +1666,15 @@
         <v>168</v>
       </c>
       <c r="I15" s="4">
-        <f>B15*0.07</f>
+        <f t="shared" si="0"/>
         <v>53167.520000000004</v>
       </c>
       <c r="J15" s="5">
-        <f>(B15*0.013)</f>
+        <f t="shared" si="1"/>
         <v>9873.9679999999989</v>
       </c>
       <c r="K15" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>63041.488000000005</v>
       </c>
       <c r="L15">
@@ -1637,15 +1710,15 @@
         <v>250</v>
       </c>
       <c r="I16" s="4">
-        <f>B16*0.07</f>
+        <f t="shared" si="0"/>
         <v>61394.060000000005</v>
       </c>
       <c r="J16" s="5">
-        <f>(B16*0.013)</f>
+        <f t="shared" si="1"/>
         <v>11401.753999999999</v>
       </c>
       <c r="K16" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>72795.813999999998</v>
       </c>
       <c r="L16">
@@ -1681,15 +1754,15 @@
         <v>255</v>
       </c>
       <c r="I17" s="4">
-        <f>B17*0.07</f>
+        <f t="shared" si="0"/>
         <v>59365.950000000004</v>
       </c>
       <c r="J17" s="5">
-        <f>(B17*0.013)</f>
+        <f t="shared" si="1"/>
         <v>11025.105</v>
       </c>
       <c r="K17" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>70391.055000000008</v>
       </c>
       <c r="L17">
@@ -1725,15 +1798,15 @@
         <v>254</v>
       </c>
       <c r="I18" s="4">
-        <f>B18*0.07</f>
+        <f t="shared" si="0"/>
         <v>48546.960000000006</v>
       </c>
       <c r="J18" s="5">
-        <f>(B18*0.013)</f>
+        <f t="shared" si="1"/>
         <v>9015.8639999999996</v>
       </c>
       <c r="K18" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>57562.824000000008</v>
       </c>
       <c r="L18">
@@ -1769,15 +1842,15 @@
         <v>242</v>
       </c>
       <c r="I19" s="4">
-        <f>B19*0.07</f>
+        <f t="shared" si="0"/>
         <v>42288.960000000006</v>
       </c>
       <c r="J19" s="5">
-        <f>(B19*0.013)</f>
+        <f t="shared" si="1"/>
         <v>7853.6639999999998</v>
       </c>
       <c r="K19" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>50142.624000000003</v>
       </c>
       <c r="L19">
@@ -1813,15 +1886,15 @@
         <v>309</v>
       </c>
       <c r="I20" s="4">
-        <f>B20*0.07</f>
+        <f t="shared" si="0"/>
         <v>77545.440000000002</v>
       </c>
       <c r="J20" s="5">
-        <f>(B20*0.013)</f>
+        <f t="shared" si="1"/>
         <v>14401.295999999998</v>
       </c>
       <c r="K20" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>91946.736000000004</v>
       </c>
       <c r="L20">
@@ -1857,15 +1930,15 @@
         <v>164</v>
       </c>
       <c r="I21" s="4">
-        <f>B21*0.07</f>
+        <f t="shared" si="0"/>
         <v>41893.880000000005</v>
       </c>
       <c r="J21" s="5">
-        <f>(B21*0.013)</f>
+        <f t="shared" si="1"/>
         <v>7780.2919999999995</v>
       </c>
       <c r="K21" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>49674.172000000006</v>
       </c>
       <c r="L21">
@@ -1901,15 +1974,15 @@
         <v>250</v>
       </c>
       <c r="I22" s="4">
-        <f>B22*0.07</f>
+        <f t="shared" si="0"/>
         <v>56578.48</v>
       </c>
       <c r="J22" s="5">
-        <f>(B22*0.013)</f>
+        <f t="shared" si="1"/>
         <v>10507.431999999999</v>
       </c>
       <c r="K22" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>67085.911999999997</v>
       </c>
       <c r="L22">
@@ -1945,15 +2018,15 @@
         <v>172</v>
       </c>
       <c r="I23" s="4">
-        <f>B23*0.07</f>
+        <f t="shared" si="0"/>
         <v>55297.200000000004</v>
       </c>
       <c r="J23" s="5">
-        <f>(B23*0.013)</f>
+        <f t="shared" si="1"/>
         <v>10269.48</v>
       </c>
       <c r="K23" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>65566.680000000008</v>
       </c>
       <c r="L23">
@@ -1985,19 +2058,19 @@
       <c r="G24" s="2">
         <v>642</v>
       </c>
-      <c r="H24" s="9">
+      <c r="H24" s="8">
         <v>47</v>
       </c>
       <c r="I24" s="4">
-        <f>B24*0.07</f>
+        <f t="shared" si="0"/>
         <v>67275.180000000008</v>
       </c>
       <c r="J24" s="5">
-        <f>(B24*0.013)</f>
+        <f t="shared" si="1"/>
         <v>12493.962</v>
       </c>
       <c r="K24" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>79769.142000000007</v>
       </c>
       <c r="L24">
@@ -2007,9 +2080,977 @@
         <v>11</v>
       </c>
     </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A25" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="B25" s="10">
+        <v>784027</v>
+      </c>
+      <c r="C25" s="8">
+        <v>1313</v>
+      </c>
+      <c r="D25" s="11">
+        <v>1307</v>
+      </c>
+      <c r="E25" s="8">
+        <v>153</v>
+      </c>
+      <c r="F25" s="2">
+        <v>114</v>
+      </c>
+      <c r="G25" s="2">
+        <v>613</v>
+      </c>
+      <c r="H25" s="2">
+        <v>287</v>
+      </c>
+      <c r="I25" s="12">
+        <f t="shared" ref="I25:I46" si="3">B25*0.07</f>
+        <v>54881.890000000007</v>
+      </c>
+      <c r="J25" s="13">
+        <f t="shared" ref="J25:J46" si="4">(B25*0.013)</f>
+        <v>10192.350999999999</v>
+      </c>
+      <c r="K25" s="14">
+        <f>I25+J25</f>
+        <v>65074.241000000009</v>
+      </c>
+      <c r="L25" s="23">
+        <v>2025</v>
+      </c>
+      <c r="M25" s="23">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A26" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="B26" s="10">
+        <v>679130</v>
+      </c>
+      <c r="C26" s="8">
+        <v>1133</v>
+      </c>
+      <c r="D26" s="11">
+        <v>1104</v>
+      </c>
+      <c r="E26" s="8">
+        <v>81</v>
+      </c>
+      <c r="F26" s="2">
+        <v>102</v>
+      </c>
+      <c r="G26" s="2">
+        <v>601</v>
+      </c>
+      <c r="H26" s="2">
+        <v>198</v>
+      </c>
+      <c r="I26" s="12">
+        <f t="shared" si="3"/>
+        <v>47539.100000000006</v>
+      </c>
+      <c r="J26" s="13">
+        <f t="shared" si="4"/>
+        <v>8828.6899999999987</v>
+      </c>
+      <c r="K26" s="14">
+        <f t="shared" ref="K26:K46" si="5">I26+J26</f>
+        <v>56367.790000000008</v>
+      </c>
+      <c r="L26" s="23">
+        <v>2025</v>
+      </c>
+      <c r="M26" s="23">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A27" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="B27" s="10">
+        <v>840360</v>
+      </c>
+      <c r="C27" s="8">
+        <v>1317</v>
+      </c>
+      <c r="D27" s="11">
+        <v>1302</v>
+      </c>
+      <c r="E27" s="8">
+        <v>106</v>
+      </c>
+      <c r="F27" s="2">
+        <v>182</v>
+      </c>
+      <c r="G27" s="2">
+        <v>596</v>
+      </c>
+      <c r="H27" s="2">
+        <v>226</v>
+      </c>
+      <c r="I27" s="12">
+        <f t="shared" si="3"/>
+        <v>58825.200000000004</v>
+      </c>
+      <c r="J27" s="13">
+        <f t="shared" si="4"/>
+        <v>10924.68</v>
+      </c>
+      <c r="K27" s="14">
+        <f t="shared" si="5"/>
+        <v>69749.88</v>
+      </c>
+      <c r="L27" s="23">
+        <v>2025</v>
+      </c>
+      <c r="M27" s="23">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A28" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B28" s="10">
+        <v>795739</v>
+      </c>
+      <c r="C28" s="8">
+        <v>1302</v>
+      </c>
+      <c r="D28" s="11">
+        <v>1316</v>
+      </c>
+      <c r="E28" s="8">
+        <v>107</v>
+      </c>
+      <c r="F28" s="2">
+        <v>121</v>
+      </c>
+      <c r="G28" s="2">
+        <v>589</v>
+      </c>
+      <c r="H28" s="2">
+        <v>225</v>
+      </c>
+      <c r="I28" s="12">
+        <f t="shared" si="3"/>
+        <v>55701.73</v>
+      </c>
+      <c r="J28" s="13">
+        <f t="shared" si="4"/>
+        <v>10344.607</v>
+      </c>
+      <c r="K28" s="14">
+        <f t="shared" si="5"/>
+        <v>66046.337</v>
+      </c>
+      <c r="L28" s="23">
+        <v>2025</v>
+      </c>
+      <c r="M28" s="23">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A29" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B29" s="10">
+        <v>1124040</v>
+      </c>
+      <c r="C29" s="8">
+        <v>1929</v>
+      </c>
+      <c r="D29" s="11">
+        <v>1915</v>
+      </c>
+      <c r="E29" s="8">
+        <v>158</v>
+      </c>
+      <c r="F29" s="2">
+        <v>188</v>
+      </c>
+      <c r="G29" s="2">
+        <v>580</v>
+      </c>
+      <c r="H29" s="2">
+        <v>403</v>
+      </c>
+      <c r="I29" s="12">
+        <f t="shared" si="3"/>
+        <v>78682.8</v>
+      </c>
+      <c r="J29" s="13">
+        <f t="shared" si="4"/>
+        <v>14612.519999999999</v>
+      </c>
+      <c r="K29" s="14">
+        <f t="shared" si="5"/>
+        <v>93295.32</v>
+      </c>
+      <c r="L29" s="23">
+        <v>2025</v>
+      </c>
+      <c r="M29" s="23">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A30" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B30" s="10">
+        <v>743862</v>
+      </c>
+      <c r="C30" s="8">
+        <v>1187</v>
+      </c>
+      <c r="D30" s="11">
+        <v>1172</v>
+      </c>
+      <c r="E30" s="8">
+        <v>115</v>
+      </c>
+      <c r="F30" s="2">
+        <v>126</v>
+      </c>
+      <c r="G30" s="2">
+        <v>597</v>
+      </c>
+      <c r="H30" s="2">
+        <v>221</v>
+      </c>
+      <c r="I30" s="12">
+        <f t="shared" si="3"/>
+        <v>52070.340000000004</v>
+      </c>
+      <c r="J30" s="13">
+        <f t="shared" si="4"/>
+        <v>9670.2060000000001</v>
+      </c>
+      <c r="K30" s="14">
+        <f t="shared" si="5"/>
+        <v>61740.546000000002</v>
+      </c>
+      <c r="L30" s="23">
+        <v>2025</v>
+      </c>
+      <c r="M30" s="23">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A31" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="B31" s="10">
+        <v>668627</v>
+      </c>
+      <c r="C31" s="8">
+        <v>1028</v>
+      </c>
+      <c r="D31" s="11">
+        <v>1048</v>
+      </c>
+      <c r="E31" s="8">
+        <v>170</v>
+      </c>
+      <c r="F31" s="2">
+        <v>128</v>
+      </c>
+      <c r="G31" s="2">
+        <v>629</v>
+      </c>
+      <c r="H31" s="2">
+        <v>236</v>
+      </c>
+      <c r="I31" s="12">
+        <f t="shared" si="3"/>
+        <v>46803.890000000007</v>
+      </c>
+      <c r="J31" s="13">
+        <f t="shared" si="4"/>
+        <v>8692.1509999999998</v>
+      </c>
+      <c r="K31" s="14">
+        <f t="shared" si="5"/>
+        <v>55496.041000000005</v>
+      </c>
+      <c r="L31" s="23">
+        <v>2025</v>
+      </c>
+      <c r="M31" s="23">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A32" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B32" s="10">
+        <v>936600</v>
+      </c>
+      <c r="C32" s="8">
+        <v>1626</v>
+      </c>
+      <c r="D32" s="11">
+        <v>1505</v>
+      </c>
+      <c r="E32" s="8">
+        <v>126</v>
+      </c>
+      <c r="F32" s="2">
+        <v>202</v>
+      </c>
+      <c r="G32" s="2">
+        <v>600</v>
+      </c>
+      <c r="H32" s="2">
+        <v>419</v>
+      </c>
+      <c r="I32" s="12">
+        <f t="shared" si="3"/>
+        <v>65562</v>
+      </c>
+      <c r="J32" s="13">
+        <f t="shared" si="4"/>
+        <v>12175.8</v>
+      </c>
+      <c r="K32" s="14">
+        <f t="shared" si="5"/>
+        <v>77737.8</v>
+      </c>
+      <c r="L32" s="23">
+        <v>2025</v>
+      </c>
+      <c r="M32" s="23">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A33" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B33" s="10">
+        <v>1595392</v>
+      </c>
+      <c r="C33" s="8">
+        <v>2291</v>
+      </c>
+      <c r="D33" s="11">
+        <v>2257</v>
+      </c>
+      <c r="E33" s="8">
+        <v>258</v>
+      </c>
+      <c r="F33" s="2">
+        <v>304</v>
+      </c>
+      <c r="G33" s="2">
+        <v>656</v>
+      </c>
+      <c r="H33" s="2">
+        <v>526</v>
+      </c>
+      <c r="I33" s="12">
+        <f t="shared" si="3"/>
+        <v>111677.44000000002</v>
+      </c>
+      <c r="J33" s="13">
+        <f t="shared" si="4"/>
+        <v>20740.095999999998</v>
+      </c>
+      <c r="K33" s="14">
+        <f t="shared" si="5"/>
+        <v>132417.53600000002</v>
+      </c>
+      <c r="L33" s="23">
+        <v>2025</v>
+      </c>
+      <c r="M33" s="23">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A34" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B34" s="10">
+        <v>402441</v>
+      </c>
+      <c r="C34" s="8">
+        <v>608</v>
+      </c>
+      <c r="D34" s="11">
+        <v>618</v>
+      </c>
+      <c r="E34" s="8">
+        <v>97</v>
+      </c>
+      <c r="F34" s="2">
+        <v>83</v>
+      </c>
+      <c r="G34" s="2">
+        <v>607</v>
+      </c>
+      <c r="H34" s="2">
+        <v>154</v>
+      </c>
+      <c r="I34" s="12">
+        <f t="shared" si="3"/>
+        <v>28170.870000000003</v>
+      </c>
+      <c r="J34" s="13">
+        <f t="shared" si="4"/>
+        <v>5231.7330000000002</v>
+      </c>
+      <c r="K34" s="14">
+        <f t="shared" si="5"/>
+        <v>33402.603000000003</v>
+      </c>
+      <c r="L34" s="23">
+        <v>2025</v>
+      </c>
+      <c r="M34" s="23">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A35" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="B35" s="10">
+        <v>1132285</v>
+      </c>
+      <c r="C35" s="8">
+        <v>1850</v>
+      </c>
+      <c r="D35" s="11">
+        <v>1818</v>
+      </c>
+      <c r="E35" s="8">
+        <v>177</v>
+      </c>
+      <c r="F35" s="2">
+        <v>182</v>
+      </c>
+      <c r="G35" s="2">
+        <v>595</v>
+      </c>
+      <c r="H35" s="2">
+        <v>391</v>
+      </c>
+      <c r="I35" s="12">
+        <f t="shared" si="3"/>
+        <v>79259.950000000012</v>
+      </c>
+      <c r="J35" s="13">
+        <f t="shared" si="4"/>
+        <v>14719.705</v>
+      </c>
+      <c r="K35" s="14">
+        <f t="shared" si="5"/>
+        <v>93979.655000000013</v>
+      </c>
+      <c r="L35" s="23">
+        <v>2025</v>
+      </c>
+      <c r="M35" s="23">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A36" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B36" s="10">
+        <v>1092854</v>
+      </c>
+      <c r="C36" s="8">
+        <v>1665</v>
+      </c>
+      <c r="D36" s="11">
+        <v>1637</v>
+      </c>
+      <c r="E36" s="8">
+        <v>164</v>
+      </c>
+      <c r="F36" s="2">
+        <v>168</v>
+      </c>
+      <c r="G36" s="2">
+        <v>622</v>
+      </c>
+      <c r="H36" s="2">
+        <v>377</v>
+      </c>
+      <c r="I36" s="12">
+        <f t="shared" si="3"/>
+        <v>76499.780000000013</v>
+      </c>
+      <c r="J36" s="13">
+        <f t="shared" si="4"/>
+        <v>14207.101999999999</v>
+      </c>
+      <c r="K36" s="14">
+        <f t="shared" si="5"/>
+        <v>90706.882000000012</v>
+      </c>
+      <c r="L36" s="23">
+        <v>2025</v>
+      </c>
+      <c r="M36" s="23">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A37" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B37" s="10">
+        <v>759536</v>
+      </c>
+      <c r="C37" s="8">
+        <v>1176</v>
+      </c>
+      <c r="D37" s="11">
+        <v>1245</v>
+      </c>
+      <c r="E37" s="8">
+        <v>132</v>
+      </c>
+      <c r="F37" s="2">
+        <v>123</v>
+      </c>
+      <c r="G37" s="2">
+        <v>592</v>
+      </c>
+      <c r="H37" s="2">
+        <v>168</v>
+      </c>
+      <c r="I37" s="12">
+        <f t="shared" si="3"/>
+        <v>53167.520000000004</v>
+      </c>
+      <c r="J37" s="13">
+        <f t="shared" si="4"/>
+        <v>9873.9679999999989</v>
+      </c>
+      <c r="K37" s="14">
+        <f t="shared" si="5"/>
+        <v>63041.488000000005</v>
+      </c>
+      <c r="L37" s="23">
+        <v>2025</v>
+      </c>
+      <c r="M37" s="23">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A38" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="B38" s="10">
+        <v>877058</v>
+      </c>
+      <c r="C38" s="8">
+        <v>1613</v>
+      </c>
+      <c r="D38" s="11">
+        <v>1597</v>
+      </c>
+      <c r="E38" s="8">
+        <v>120</v>
+      </c>
+      <c r="F38" s="2">
+        <v>159</v>
+      </c>
+      <c r="G38" s="2">
+        <v>553</v>
+      </c>
+      <c r="H38" s="2">
+        <v>250</v>
+      </c>
+      <c r="I38" s="12">
+        <f t="shared" si="3"/>
+        <v>61394.060000000005</v>
+      </c>
+      <c r="J38" s="13">
+        <f t="shared" si="4"/>
+        <v>11401.753999999999</v>
+      </c>
+      <c r="K38" s="14">
+        <f t="shared" si="5"/>
+        <v>72795.813999999998</v>
+      </c>
+      <c r="L38" s="23">
+        <v>2025</v>
+      </c>
+      <c r="M38" s="23">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="39" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A39" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B39" s="10">
+        <v>848085</v>
+      </c>
+      <c r="C39" s="8">
+        <v>1411</v>
+      </c>
+      <c r="D39" s="11">
+        <v>1396</v>
+      </c>
+      <c r="E39" s="8">
+        <v>116</v>
+      </c>
+      <c r="F39" s="2">
+        <v>147</v>
+      </c>
+      <c r="G39" s="2">
+        <v>591</v>
+      </c>
+      <c r="H39" s="2">
+        <v>255</v>
+      </c>
+      <c r="I39" s="12">
+        <f t="shared" si="3"/>
+        <v>59365.950000000004</v>
+      </c>
+      <c r="J39" s="13">
+        <f t="shared" si="4"/>
+        <v>11025.105</v>
+      </c>
+      <c r="K39" s="14">
+        <f t="shared" si="5"/>
+        <v>70391.055000000008</v>
+      </c>
+      <c r="L39" s="23">
+        <v>2025</v>
+      </c>
+      <c r="M39" s="23">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="40" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A40" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="B40" s="10">
+        <v>693528</v>
+      </c>
+      <c r="C40" s="8">
+        <v>1209</v>
+      </c>
+      <c r="D40" s="11">
+        <v>1172</v>
+      </c>
+      <c r="E40" s="8">
+        <v>101</v>
+      </c>
+      <c r="F40" s="2">
+        <v>101</v>
+      </c>
+      <c r="G40" s="2">
+        <v>568</v>
+      </c>
+      <c r="H40" s="2">
+        <v>254</v>
+      </c>
+      <c r="I40" s="12">
+        <f t="shared" si="3"/>
+        <v>48546.960000000006</v>
+      </c>
+      <c r="J40" s="13">
+        <f t="shared" si="4"/>
+        <v>9015.8639999999996</v>
+      </c>
+      <c r="K40" s="14">
+        <f t="shared" si="5"/>
+        <v>57562.824000000008</v>
+      </c>
+      <c r="L40" s="23">
+        <v>2025</v>
+      </c>
+      <c r="M40" s="23">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="41" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A41" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B41" s="10">
+        <v>604128</v>
+      </c>
+      <c r="C41" s="8">
+        <v>1015</v>
+      </c>
+      <c r="D41" s="11">
+        <v>991</v>
+      </c>
+      <c r="E41" s="8">
+        <v>106</v>
+      </c>
+      <c r="F41" s="2">
+        <v>106</v>
+      </c>
+      <c r="G41" s="2">
+        <v>609</v>
+      </c>
+      <c r="H41" s="2">
+        <v>242</v>
+      </c>
+      <c r="I41" s="12">
+        <f t="shared" si="3"/>
+        <v>42288.960000000006</v>
+      </c>
+      <c r="J41" s="13">
+        <f t="shared" si="4"/>
+        <v>7853.6639999999998</v>
+      </c>
+      <c r="K41" s="14">
+        <f t="shared" si="5"/>
+        <v>50142.624000000003</v>
+      </c>
+      <c r="L41" s="23">
+        <v>2025</v>
+      </c>
+      <c r="M41" s="23">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="42" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A42" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B42" s="10">
+        <v>1107792</v>
+      </c>
+      <c r="C42" s="8">
+        <v>1707</v>
+      </c>
+      <c r="D42" s="11">
+        <v>1706</v>
+      </c>
+      <c r="E42" s="8">
+        <v>155</v>
+      </c>
+      <c r="F42" s="2">
+        <v>149</v>
+      </c>
+      <c r="G42" s="2">
+        <v>628</v>
+      </c>
+      <c r="H42" s="2">
+        <v>309</v>
+      </c>
+      <c r="I42" s="12">
+        <f t="shared" si="3"/>
+        <v>77545.440000000002</v>
+      </c>
+      <c r="J42" s="13">
+        <f t="shared" si="4"/>
+        <v>14401.295999999998</v>
+      </c>
+      <c r="K42" s="14">
+        <f t="shared" si="5"/>
+        <v>91946.736000000004</v>
+      </c>
+      <c r="L42" s="23">
+        <v>2025</v>
+      </c>
+      <c r="M42" s="23">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="43" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A43" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B43" s="10">
+        <v>598484</v>
+      </c>
+      <c r="C43" s="8">
+        <v>846</v>
+      </c>
+      <c r="D43" s="11">
+        <v>887</v>
+      </c>
+      <c r="E43" s="8">
+        <v>129</v>
+      </c>
+      <c r="F43" s="2">
+        <v>101</v>
+      </c>
+      <c r="G43" s="2">
+        <v>628</v>
+      </c>
+      <c r="H43" s="2">
+        <v>164</v>
+      </c>
+      <c r="I43" s="12">
+        <f t="shared" si="3"/>
+        <v>41893.880000000005</v>
+      </c>
+      <c r="J43" s="13">
+        <f t="shared" si="4"/>
+        <v>7780.2919999999995</v>
+      </c>
+      <c r="K43" s="14">
+        <f t="shared" si="5"/>
+        <v>49674.172000000006</v>
+      </c>
+      <c r="L43" s="23">
+        <v>2025</v>
+      </c>
+      <c r="M43" s="23">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="44" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A44" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="B44" s="10">
+        <v>808264</v>
+      </c>
+      <c r="C44" s="8">
+        <v>1380</v>
+      </c>
+      <c r="D44" s="11">
+        <v>1376</v>
+      </c>
+      <c r="E44" s="8">
+        <v>142</v>
+      </c>
+      <c r="F44" s="2">
+        <v>98</v>
+      </c>
+      <c r="G44" s="2">
+        <v>568</v>
+      </c>
+      <c r="H44" s="2">
+        <v>250</v>
+      </c>
+      <c r="I44" s="12">
+        <f t="shared" si="3"/>
+        <v>56578.48</v>
+      </c>
+      <c r="J44" s="13">
+        <f t="shared" si="4"/>
+        <v>10507.431999999999</v>
+      </c>
+      <c r="K44" s="14">
+        <f t="shared" si="5"/>
+        <v>67085.911999999997</v>
+      </c>
+      <c r="L44" s="23">
+        <v>2025</v>
+      </c>
+      <c r="M44" s="23">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A45" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B45" s="10">
+        <v>789960</v>
+      </c>
+      <c r="C45" s="8">
+        <v>1131</v>
+      </c>
+      <c r="D45" s="11">
+        <v>1123</v>
+      </c>
+      <c r="E45" s="8">
+        <v>115</v>
+      </c>
+      <c r="F45" s="2">
+        <v>137</v>
+      </c>
+      <c r="G45" s="2">
+        <v>681</v>
+      </c>
+      <c r="H45" s="2">
+        <v>172</v>
+      </c>
+      <c r="I45" s="12">
+        <f t="shared" si="3"/>
+        <v>55297.200000000004</v>
+      </c>
+      <c r="J45" s="13">
+        <f t="shared" si="4"/>
+        <v>10269.48</v>
+      </c>
+      <c r="K45" s="14">
+        <f t="shared" si="5"/>
+        <v>65566.680000000008</v>
+      </c>
+      <c r="L45" s="23">
+        <v>2025</v>
+      </c>
+      <c r="M45" s="23">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="46" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A46" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="B46" s="16">
+        <v>961074</v>
+      </c>
+      <c r="C46" s="17">
+        <v>1462</v>
+      </c>
+      <c r="D46" s="18">
+        <v>1686</v>
+      </c>
+      <c r="E46" s="17">
+        <v>315</v>
+      </c>
+      <c r="F46" s="19">
+        <v>1</v>
+      </c>
+      <c r="G46" s="19">
+        <v>642</v>
+      </c>
+      <c r="H46" s="19">
+        <v>47</v>
+      </c>
+      <c r="I46" s="20">
+        <f t="shared" si="3"/>
+        <v>67275.180000000008</v>
+      </c>
+      <c r="J46" s="21">
+        <f t="shared" si="4"/>
+        <v>12493.962</v>
+      </c>
+      <c r="K46" s="22">
+        <f t="shared" si="5"/>
+        <v>79769.142000000007</v>
+      </c>
+      <c r="L46" s="23">
+        <v>2025</v>
+      </c>
+      <c r="M46" s="23">
+        <v>12</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="B3:B24">
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="lessThan">
+  <conditionalFormatting sqref="B3:B46">
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="lessThan">
       <formula>10020</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>